<commit_message>
Layout atualizado, tudo funcionando
</commit_message>
<xml_diff>
--- a/Planilha Mensal - eliminados registros de ex líderes.xlsx
+++ b/Planilha Mensal - eliminados registros de ex líderes.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTA_TESTE_K_102814" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LISTA_TESTE_K_102814" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LISTA_TESTE_K_102814'!$A$1:$I$1</definedName>

</xml_diff>